<commit_message>
Catalog: BR3791 + BR4158 (BR3791-Master family) moved to Discontinued; Discontinued tab hidden
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/automation/catalog.xlsx
+++ b/automation/catalog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Discontinued" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M212"/>
+  <dimension ref="A1:M210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7335,26 +7335,26 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>BR3791</t>
+          <t>KT8153</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>B077ZFT4YF</t>
+          <t>B07FT1LP8R</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>BR3791_FBA</t>
+          <t>KT8153_FBA</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>BR3791-Master</t>
+          <t>KT8153-Master</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7389,26 +7389,26 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>BR4158</t>
+          <t>KT8100</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>B07Q262HDG</t>
+          <t>B0742QYGGN</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>BR4158_FBA</t>
+          <t>KT8100_FBA</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>BR3791-Master</t>
+          <t>KT8100-Master</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7443,26 +7443,26 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>KT8153</t>
+          <t>BR4238</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>B07FT1LP8R</t>
+          <t>B0B78BR6NM</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>KT8153_FBA</t>
+          <t>BR4238_FBA</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>KT8153-Master</t>
+          <t>KT8100-Master</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7497,26 +7497,26 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>KT8100</t>
+          <t>BN1663</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>B0742QYGGN</t>
+          <t>B072PX13TJ</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>KT8100_FBA</t>
+          <t>BN1663_FBA</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>KT8100-Master</t>
+          <t>BN1663-Master</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7551,26 +7551,26 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>BR4238</t>
+          <t>BN1798</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>B0B78BR6NM</t>
+          <t>B07CT87DVQ</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>BR4238_FBA</t>
+          <t>BN1798_FBA</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>KT8100-Master</t>
+          <t>BN1798-Master</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -7605,31 +7605,31 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>BN1663</t>
+          <t>NC4297</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>B072PX13TJ</t>
+          <t>B09826V9Z8</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>BN1663_FBA</t>
+          <t>NC4297_FBA</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>BN1663-Master</t>
+          <t>NC4285-Master</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="G141" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>PJ_FJ</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="K141" t="n">
@@ -7659,31 +7659,31 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>BN1798</t>
+          <t>NC4285</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>B07CT87DVQ</t>
+          <t>B08Q2WMF25</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>BN1798_FBA</t>
+          <t>NC4285_FBA</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>BN1798-Master</t>
+          <t>NC4285-Master</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>PJ_FJ</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="K142" t="n">
@@ -7713,21 +7713,21 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>NC4297</t>
+          <t>NC4367</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>B09826V9Z8</t>
+          <t>B0BZB723JD</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>NC4297_FBA</t>
+          <t>NC4367_FBA</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -7767,21 +7767,21 @@
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>NC4285</t>
+          <t>NC4290-1</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>B08Q2WMF25</t>
+          <t>B0DGWDSSKW</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>NC4285_FBA</t>
+          <t>NC4290-1</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -7821,21 +7821,21 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>NC4367</t>
+          <t>NC4364</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>B0BZB723JD</t>
+          <t>B0BKKQ79FB</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>NC4367_FBA</t>
+          <t>NC4364_FBA</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -7875,21 +7875,21 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>NC4290-1</t>
+          <t>NC4298</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>B0DGWDSSKW</t>
+          <t>B09825NYCX</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>NC4290-1</t>
+          <t>NC4298_FBA</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -7929,21 +7929,21 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>NC4364</t>
+          <t>NC4352</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>B0BKKQ79FB</t>
+          <t>B0B73W137Q</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>NC4364_FBA</t>
+          <t>NC4352_FBA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -7983,21 +7983,21 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>NC4298</t>
+          <t>NC4303</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>B09825NYCX</t>
+          <t>B09825SRFQ</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>NC4298_FBA</t>
+          <t>NC4303_FBA</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -8037,21 +8037,21 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>NC4352</t>
+          <t>NC4379</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>B0B73W137Q</t>
+          <t>B0CDBRW16Q</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>NC4352_FBA</t>
+          <t>NC4379_FBA</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -8091,21 +8091,21 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>NC4303</t>
+          <t>NC4314</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>B09825SRFQ</t>
+          <t>B09FTQ6G3F</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>NC4303_FBA</t>
+          <t>NC4314_FBA</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -8145,21 +8145,21 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>NC4379</t>
+          <t>NC4301</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>B0CDBRW16Q</t>
+          <t>B09824YTT3</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>NC4379_FBA</t>
+          <t>NC4301_FBA</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -8199,21 +8199,21 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>NC4314</t>
+          <t>NC4380</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>B09FTQ6G3F</t>
+          <t>B0CDBRNT3H</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>NC4314_FBA</t>
+          <t>NC4380_FBA</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -8253,21 +8253,21 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>NC4301</t>
+          <t>NC4382</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>B09824YTT3</t>
+          <t>B0CPBLZTWT</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>NC4301_FBA</t>
+          <t>NC4382</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -8307,21 +8307,21 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>NC4380</t>
+          <t>NC4342</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>B0CDBRNT3H</t>
+          <t>B0B73XGZSM</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>NC4380_FBA</t>
+          <t>NC4342_FBA</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -8361,21 +8361,21 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>NC4382</t>
+          <t>NC4390</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>B0CPBLZTWT</t>
+          <t>B0H3QBP4XW</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>NC4382</t>
+          <t>NC4390</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -8415,21 +8415,21 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>NC4342</t>
+          <t>NC4394</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>B0B73XGZSM</t>
+          <t>B0H4F11HFF</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>NC4342_FBA</t>
+          <t>NC4394</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -8469,21 +8469,21 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>NC4390</t>
+          <t>NC4395</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>B0H3QBP4XW</t>
+          <t>B0H4DTWJT1</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>NC4390</t>
+          <t>NC4395</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -8523,21 +8523,21 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>NC4394</t>
+          <t>NC4396</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>B0H4F11HFF</t>
+          <t>B0H4DRS9P1</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>NC4394</t>
+          <t>NC4396</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -8577,26 +8577,26 @@
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>NC4395</t>
+          <t>NC4058</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>B0H4DTWJT1</t>
+          <t>B01HSJ3T6M</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>NC4395</t>
+          <t>NC4058_FBA</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>NC4285-Master</t>
+          <t>NC4058-Master</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -8631,26 +8631,26 @@
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>NC4396</t>
+          <t>NC4250</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>B0H4DRS9P1</t>
+          <t>B07YCX7ZF4</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>NC4396</t>
+          <t>NC4250_FBA</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>NC4285-Master</t>
+          <t>NC4058-Master</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -8685,21 +8685,21 @@
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>NC4058</t>
+          <t>NC4293</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>B01HSJ3T6M</t>
+          <t>B093FX1RJJ</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>NC4058_FBA</t>
+          <t>NC4293_FBA</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -8739,21 +8739,21 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>NC4250</t>
+          <t>NC4270</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>B07YCX7ZF4</t>
+          <t>B082LRFT53</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>NC4250_FBA</t>
+          <t>NC4270_FBA</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -8793,21 +8793,21 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>NC4293</t>
+          <t>NC4377</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>B093FX1RJJ</t>
+          <t>B0CCRK55BW</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>NC4293_FBA</t>
+          <t>NC4377_FBA</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -8847,21 +8847,21 @@
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>NC4270</t>
+          <t>NC4275</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>B082LRFT53</t>
+          <t>B082LVZWGW</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>NC4270_FBA</t>
+          <t>NC4275_FBA</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -8901,21 +8901,21 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>NC4377</t>
+          <t>NC4274</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>B0CCRK55BW</t>
+          <t>B082LMV5P7</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>NC4377_FBA</t>
+          <t>NC4274_FBA</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -8955,21 +8955,21 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>NC4275</t>
+          <t>NC4272</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>B082LVZWGW</t>
+          <t>B082LN9HQ3</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>NC4275_FBA</t>
+          <t>NC4272_FBA</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -9009,21 +9009,21 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>NC4274</t>
+          <t>NC4273</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>B082LMV5P7</t>
+          <t>B082LMC563</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>NC4274_FBA</t>
+          <t>NC4273_FBA</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -9063,26 +9063,26 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>NC4272</t>
+          <t>NC4059-1</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>B082LN9HQ3</t>
+          <t>B0DDT2L7FL</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>NC4272_FBA</t>
+          <t>NC4059-1</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>NC4058-Master</t>
+          <t>NC4059-Master</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -9117,26 +9117,26 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>NC4273</t>
+          <t>NC4305</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>B082LMC563</t>
+          <t>B0988741SV</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>NC4273_FBA</t>
+          <t>NC4305_FBA</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>NC4058-Master</t>
+          <t>NC4059-Master</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -9171,21 +9171,21 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>NC4059-1</t>
+          <t>NC4084-1</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>B0DDT2L7FL</t>
+          <t>B07WNRW3SV</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>NC4059-1</t>
+          <t>NC4084-1_FBA</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -9225,21 +9225,21 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>NC4305</t>
+          <t>NC4284</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>B0988741SV</t>
+          <t>B08Q31XC28</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>NC4305_FBA</t>
+          <t>NC4284_FBA</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -9279,21 +9279,21 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>NC4084-1</t>
+          <t>NC4103</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>B07WNRW3SV</t>
+          <t>B01M99D9CI</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>NC4084-1_FBA</t>
+          <t>NC4103_FBA</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -9333,21 +9333,21 @@
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>NC4284</t>
+          <t>NC4381</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>B08Q31XC28</t>
+          <t>B0CKXVDSXT</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>NC4284_FBA</t>
+          <t>NC4381</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -9387,21 +9387,21 @@
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>NC4103</t>
+          <t>NC4353</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>B01M99D9CI</t>
+          <t>B0B7KQLMYN</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>NC4103_FBA</t>
+          <t>NC4353_FBA</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -9441,21 +9441,21 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>NC4381</t>
+          <t>NC4059</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>B0CKXVDSXT</t>
+          <t>B01IACWDOK</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>NC4381</t>
+          <t>NC4059_FBA</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -9495,26 +9495,26 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>NC4353</t>
+          <t>NC4386-1</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>B0B7KQLMYN</t>
+          <t>B0DGWFF5QS</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>NC4353_FBA</t>
+          <t>NC4386-1</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>NC4059-Master</t>
+          <t>NC4329-Master</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -9549,26 +9549,26 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>NC4059</t>
+          <t>NC4179</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>B01IACWDOK</t>
+          <t>B01MZYSIP1</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>NC4059_FBA</t>
+          <t>NC4179_FBA</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>NC4059-Master</t>
+          <t>NC4085-Master</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -9603,26 +9603,26 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>NC4386-1</t>
+          <t>NC4085-1</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>B0DGWFF5QS</t>
+          <t>B0DDT2TSPK</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>NC4386-1</t>
+          <t>NC4085-1</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>NC4329-Master</t>
+          <t>NC4085-Master</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -9657,21 +9657,21 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>NC4179</t>
+          <t>NC4247</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>B01MZYSIP1</t>
+          <t>B07WFHXKGM</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>NC4179_FBA</t>
+          <t>NC4247_FBA</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -9711,21 +9711,21 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>NC4085-1</t>
+          <t>NC4294</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>B0DDT2TSPK</t>
+          <t>B093FWLTX3</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>NC4085-1</t>
+          <t>NC4294_FBA</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -9765,21 +9765,21 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>NC4247</t>
+          <t>NC4340</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>B07WFHXKGM</t>
+          <t>B0B6H8T4GK</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>NC4247_FBA</t>
+          <t>NC4340_FBA</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -9819,21 +9819,21 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>NC4294</t>
+          <t>NC4276</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>B093FWLTX3</t>
+          <t>B082MTZ58T</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>NC4294_FBA</t>
+          <t>NC4276_FBA</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -9873,26 +9873,26 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>NC4340</t>
+          <t>NC4388</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>B0B6H8T4GK</t>
+          <t>B0CYLGPQVS</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>NC4340_FBA</t>
+          <t>NC4388</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>NC4085-Master</t>
+          <t>NC4256-Master</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -9927,26 +9927,26 @@
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>NC4276</t>
+          <t>NC4389</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>B082MTZ58T</t>
+          <t>B0D4DXYK1X</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>NC4276_FBA</t>
+          <t>NC4389</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>NC4085-Master</t>
+          <t>NC4256-Master</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -9981,26 +9981,26 @@
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>NC4388</t>
+          <t>NC4400-A</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>B0CYLGPQVS</t>
+          <t>B0DJSWD9YL</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>NC4388</t>
+          <t>NC4400-A</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>NC4256-Master</t>
+          <t>NC4400-Master</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -10035,26 +10035,26 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>NC4389</t>
+          <t>NC4400-B</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>B0D4DXYK1X</t>
+          <t>B0DJSYMJ3Y</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>NC4389</t>
+          <t>NC4400-B</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>NC4256-Master</t>
+          <t>NC4400-Master</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -10089,21 +10089,21 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>NC4400-A</t>
+          <t>NC4400-C</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>B0DJSWD9YL</t>
+          <t>B0DJSZ6BC4</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>NC4400-A</t>
+          <t>NC4400-C</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -10143,21 +10143,21 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>NC4400-B</t>
+          <t>NC4400-D</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>B0DJSYMJ3Y</t>
+          <t>B0DJSXMVW3</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>NC4400-B</t>
+          <t>NC4400-D</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -10197,21 +10197,21 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>NC4400-C</t>
+          <t>NC4400-E</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>B0DJSZ6BC4</t>
+          <t>B0DJSXTMB1</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>NC4400-C</t>
+          <t>NC4400-E</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -10251,21 +10251,21 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>NC4400-D</t>
+          <t>NC4400-F</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>B0DJSXMVW3</t>
+          <t>B0DJVQQ2C7</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>NC4400-D</t>
+          <t>NC4400-F</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -10305,21 +10305,21 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>NC4400-E</t>
+          <t>NC4400-G</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>B0DJSXTMB1</t>
+          <t>B0DJSX9JPJ</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>NC4400-E</t>
+          <t>NC4400-G</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -10359,21 +10359,21 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>NC4400-F</t>
+          <t>NC4400-H</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>B0DJVQQ2C7</t>
+          <t>B0DJSXXKS8</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>NC4400-F</t>
+          <t>NC4400-H</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -10413,21 +10413,21 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>NC4400-G</t>
+          <t>NC4400-I</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>B0DJSX9JPJ</t>
+          <t>B0DJVQZ5ZG</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>NC4400-G</t>
+          <t>NC4400-I</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -10467,21 +10467,21 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>NC4400-H</t>
+          <t>NC4400-J</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>B0DJSXXKS8</t>
+          <t>B0DJSXL9PC</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>NC4400-H</t>
+          <t>NC4400-J</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -10521,21 +10521,21 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>NC4400-I</t>
+          <t>NC4400-K1</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>B0DJVQZ5ZG</t>
+          <t>B0FHKHJ82B</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>NC4400-I</t>
+          <t>NC4400-K1</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -10575,21 +10575,21 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>NC4400-J</t>
+          <t>NC4400-L1</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>B0DJSXL9PC</t>
+          <t>B0FJ1Z3LVM</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>NC4400-J</t>
+          <t>NC4400-L1</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -10629,21 +10629,21 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>NC4400-K1</t>
+          <t>NC4400-M</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>B0FHKHJ82B</t>
+          <t>B0DJSW8HC8</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>NC4400-K1</t>
+          <t>NC4400-M</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -10683,21 +10683,21 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>NC4400-L1</t>
+          <t>NC4400-N</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>B0FJ1Z3LVM</t>
+          <t>B0DJVRPM41</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>NC4400-L1</t>
+          <t>NC4400-N</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -10737,21 +10737,21 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>NC4400-M</t>
+          <t>NC4400-O</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>B0DJSW8HC8</t>
+          <t>B0DJVQCN8T</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>NC4400-M</t>
+          <t>NC4400-O</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -10791,21 +10791,21 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>NC4400-N</t>
+          <t>NC4400-P</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>B0DJVRPM41</t>
+          <t>B0DJSXS41D</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>NC4400-N</t>
+          <t>NC4400-P</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -10845,21 +10845,21 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>NC4400-O</t>
+          <t>NC4400-Q</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>B0DJVQCN8T</t>
+          <t>B0DJVSFZMJ</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>NC4400-O</t>
+          <t>NC4400-Q</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -10899,21 +10899,21 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>NC4400-P</t>
+          <t>NC4400-R</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>B0DJSXS41D</t>
+          <t>B0DJSX3V6P</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>NC4400-P</t>
+          <t>NC4400-R</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -10953,21 +10953,21 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>NC4400-Q</t>
+          <t>NC4400-S</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>B0DJVSFZMJ</t>
+          <t>B0DJSX3BG2</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>NC4400-Q</t>
+          <t>NC4400-S</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -11007,21 +11007,21 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>NC4400-R</t>
+          <t>NC4400-T</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>B0DJSX3V6P</t>
+          <t>B0DJSWBSBS</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>NC4400-R</t>
+          <t>NC4400-T</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -11061,21 +11061,21 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>NC4400-S</t>
+          <t>NC4400-U</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>B0DJSX3BG2</t>
+          <t>B0DJVRDW13</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>NC4400-S</t>
+          <t>NC4400-U</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -11115,21 +11115,21 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>NC4400-T</t>
+          <t>NC4400-V</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>B0DJSWBSBS</t>
+          <t>B0DJSXXDKR</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>NC4400-T</t>
+          <t>NC4400-V</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -11169,21 +11169,21 @@
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>NC4400-U</t>
+          <t>NC4400-W</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>B0DJVRDW13</t>
+          <t>B0DJVQ34DH</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>NC4400-U</t>
+          <t>NC4400-W</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -11223,21 +11223,21 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>NC4400-V</t>
+          <t>NC4400-X</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>B0DJSXXDKR</t>
+          <t>B0DJVRS3S2</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>NC4400-V</t>
+          <t>NC4400-X</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -11277,21 +11277,21 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>NC4400-W</t>
+          <t>NC4400-Y</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>B0DJVQ34DH</t>
+          <t>B0DJVNLV9V</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>NC4400-W</t>
+          <t>NC4400-Y</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -11331,21 +11331,21 @@
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>NC4400-X</t>
+          <t>NC4400-Z</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>B0DJVRS3S2</t>
+          <t>B0DJVQSFLW</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>NC4400-X</t>
+          <t>NC4400-Z</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -11380,114 +11380,6 @@
         <v>30</v>
       </c>
       <c r="L210" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>210</v>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>NC4400-Y</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>B0DJVNLV9V</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>NC4400-Y</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>NC4400-Master</t>
-        </is>
-      </c>
-      <c r="F211" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="G211" t="n">
-        <v>3</v>
-      </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>China direct</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="J211" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="K211" t="n">
-        <v>30</v>
-      </c>
-      <c r="L211" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>211</v>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>NC4400-Z</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>B0DJVQSFLW</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>NC4400-Z</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>NC4400-Master</t>
-        </is>
-      </c>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="G212" t="n">
-        <v>3</v>
-      </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>China direct</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="J212" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="K212" t="n">
-        <v>30</v>
-      </c>
-      <c r="L212" t="n">
         <v>45</v>
       </c>
     </row>
@@ -11502,7 +11394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13541,6 +13433,50 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>B077ZFT4YF</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BR3791-Master</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BR3791_FBA</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>B07Q262HDG</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BR3791-Master</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>BR4158_FBA</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>